<commit_message>
added new assets for the running game
</commit_message>
<xml_diff>
--- a/1_SPEC/game_art_src/runner_voice/runner_vo_manifest.xlsx
+++ b/1_SPEC/game_art_src/runner_voice/runner_vo_manifest.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recording spec" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VO Manifest'!$A$4:$I$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VO Manifest'!$A$4:$I$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -70,7 +70,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -84,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00E6F4F1"/>
       </patternFill>
     </fill>
     <fill>
@@ -110,6 +110,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF8DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4ECF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -238,6 +243,24 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -611,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1048,7 @@
       <c r="F13" s="22" t="inlineStr"/>
       <c r="G13" s="23" t="inlineStr">
         <is>
-          <t>Child runs into the orb with the wrong word (1st of 3 lines).</t>
+          <t>Child runs into the orb with the wrong word. The pair then comes back.</t>
         </is>
       </c>
       <c r="H13" s="19" t="n">
@@ -1064,15 +1087,15 @@
       <c r="F14" s="22" t="inlineStr"/>
       <c r="G14" s="23" t="inlineStr">
         <is>
-          <t>After «फिर से देखिए।» on a wrong orb, followed by the correct word of that pair (2nd of 3 lines).</t>
+          <t>NOT PLAYED since r115 - a wrong orb now says only «फिर से देखिए।»; the words are read when the pair comes back.</t>
         </is>
       </c>
       <c r="H14" s="19" t="n">
         <v>1.25</v>
       </c>
-      <c r="I14" s="20" t="inlineStr">
-        <is>
-          <t>Recorded</t>
+      <c r="I14" s="24" t="inlineStr">
+        <is>
+          <t>Recorded - not used in the game</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1286,7 @@
       </c>
       <c r="G19" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H19" s="25" t="n">
@@ -1306,7 +1329,7 @@
       </c>
       <c r="G20" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H20" s="25" t="n">
@@ -1349,7 +1372,7 @@
       </c>
       <c r="G21" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H21" s="25" t="n">
@@ -1392,7 +1415,7 @@
       </c>
       <c r="G22" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H22" s="25" t="n">
@@ -1435,7 +1458,7 @@
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H23" s="25" t="n">
@@ -1478,7 +1501,7 @@
       </c>
       <c r="G24" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H24" s="25" t="n">
@@ -1521,7 +1544,7 @@
       </c>
       <c r="G25" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H25" s="25" t="n">
@@ -1564,7 +1587,7 @@
       </c>
       <c r="G26" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H26" s="25" t="n">
@@ -1607,7 +1630,7 @@
       </c>
       <c r="G27" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H27" s="25" t="n">
@@ -1650,7 +1673,7 @@
       </c>
       <c r="G28" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H28" s="25" t="n">
@@ -1693,7 +1716,7 @@
       </c>
       <c r="G29" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H29" s="25" t="n">
@@ -1736,7 +1759,7 @@
       </c>
       <c r="G30" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H30" s="25" t="n">
@@ -1779,7 +1802,7 @@
       </c>
       <c r="G31" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H31" s="25" t="n">
@@ -1822,7 +1845,7 @@
       </c>
       <c r="G32" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H32" s="25" t="n">
@@ -1865,7 +1888,7 @@
       </c>
       <c r="G33" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H33" s="25" t="n">
@@ -1908,7 +1931,7 @@
       </c>
       <c r="G34" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H34" s="25" t="n">
@@ -1951,7 +1974,7 @@
       </c>
       <c r="G35" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H35" s="25" t="n">
@@ -1994,7 +2017,7 @@
       </c>
       <c r="G36" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H36" s="25" t="n">
@@ -2037,7 +2060,7 @@
       </c>
       <c r="G37" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H37" s="25" t="n">
@@ -2080,7 +2103,7 @@
       </c>
       <c r="G38" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H38" s="25" t="n">
@@ -2123,7 +2146,7 @@
       </c>
       <c r="G39" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H39" s="25" t="n">
@@ -2166,7 +2189,7 @@
       </c>
       <c r="G40" s="29" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H40" s="25" t="n">
@@ -2209,7 +2232,7 @@
       </c>
       <c r="G41" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H41" s="30" t="n">
@@ -2252,7 +2275,7 @@
       </c>
       <c r="G42" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H42" s="30" t="n">
@@ -2295,7 +2318,7 @@
       </c>
       <c r="G43" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H43" s="30" t="n">
@@ -2338,7 +2361,7 @@
       </c>
       <c r="G44" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H44" s="30" t="n">
@@ -2381,7 +2404,7 @@
       </c>
       <c r="G45" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H45" s="30" t="n">
@@ -2424,7 +2447,7 @@
       </c>
       <c r="G46" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H46" s="30" t="n">
@@ -2467,7 +2490,7 @@
       </c>
       <c r="G47" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H47" s="30" t="n">
@@ -2510,7 +2533,7 @@
       </c>
       <c r="G48" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H48" s="30" t="n">
@@ -2553,7 +2576,7 @@
       </c>
       <c r="G49" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H49" s="30" t="n">
@@ -2596,7 +2619,7 @@
       </c>
       <c r="G50" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H50" s="30" t="n">
@@ -2639,7 +2662,7 @@
       </c>
       <c r="G51" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H51" s="30" t="n">
@@ -2682,7 +2705,7 @@
       </c>
       <c r="G52" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H52" s="30" t="n">
@@ -2725,7 +2748,7 @@
       </c>
       <c r="G53" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H53" s="30" t="n">
@@ -2768,7 +2791,7 @@
       </c>
       <c r="G54" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H54" s="30" t="n">
@@ -2811,7 +2834,7 @@
       </c>
       <c r="G55" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H55" s="30" t="n">
@@ -2854,7 +2877,7 @@
       </c>
       <c r="G56" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H56" s="30" t="n">
@@ -2897,7 +2920,7 @@
       </c>
       <c r="G57" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H57" s="30" t="n">
@@ -2940,7 +2963,7 @@
       </c>
       <c r="G58" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H58" s="30" t="n">
@@ -2983,7 +3006,7 @@
       </c>
       <c r="G59" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H59" s="30" t="n">
@@ -3026,7 +3049,7 @@
       </c>
       <c r="G60" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H60" s="30" t="n">
@@ -3069,7 +3092,7 @@
       </c>
       <c r="G61" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H61" s="30" t="n">
@@ -3112,7 +3135,7 @@
       </c>
       <c r="G62" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H62" s="30" t="n">
@@ -3155,7 +3178,7 @@
       </c>
       <c r="G63" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H63" s="30" t="n">
@@ -3198,7 +3221,7 @@
       </c>
       <c r="G64" s="34" t="inlineStr">
         <is>
-          <t>Target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
+          <t>r115: NOT spoken before the pair is caught. When a pair comes back after ONE mistake, both its words are read (left, then right); after TWO mistakes only the right word. (Was: target word: spoken once as its pair of word orbs comes near - only the word to catch, never both portals' words. Also said after «सही शब्द है» when the child misses it.</t>
         </is>
       </c>
       <c r="H64" s="30" t="n">
@@ -3210,8 +3233,1982 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="35" t="n">
+        <v>61</v>
+      </c>
+      <c r="B65" s="36" t="inlineStr">
+        <is>
+          <t>pul_x</t>
+        </is>
+      </c>
+      <c r="C65" s="36" t="inlineStr">
+        <is>
+          <t>pul_x.ogg</t>
+        </is>
+      </c>
+      <c r="D65" s="37" t="inlineStr">
+        <is>
+          <t>पूल</t>
+        </is>
+      </c>
+      <c r="E65" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F65" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G65" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «पुल» -&gt; «पूल»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H65" s="35" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="I65" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="35" t="n">
+        <v>62</v>
+      </c>
+      <c r="B66" s="36" t="inlineStr">
+        <is>
+          <t>gud_x</t>
+        </is>
+      </c>
+      <c r="C66" s="36" t="inlineStr">
+        <is>
+          <t>gud_x.ogg</t>
+        </is>
+      </c>
+      <c r="D66" s="37" t="inlineStr">
+        <is>
+          <t>गूड़</t>
+        </is>
+      </c>
+      <c r="E66" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F66" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G66" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «गुड़» -&gt; «गूड़»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H66" s="35" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I66" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="35" t="n">
+        <v>63</v>
+      </c>
+      <c r="B67" s="36" t="inlineStr">
+        <is>
+          <t>sukh_x</t>
+        </is>
+      </c>
+      <c r="C67" s="36" t="inlineStr">
+        <is>
+          <t>sukh_x.ogg</t>
+        </is>
+      </c>
+      <c r="D67" s="37" t="inlineStr">
+        <is>
+          <t>सूख</t>
+        </is>
+      </c>
+      <c r="E67" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F67" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G67" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «सुख» -&gt; «सूख»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H67" s="35" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="I67" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="35" t="n">
+        <v>64</v>
+      </c>
+      <c r="B68" s="36" t="inlineStr">
+        <is>
+          <t>chup_x</t>
+        </is>
+      </c>
+      <c r="C68" s="36" t="inlineStr">
+        <is>
+          <t>chup_x.ogg</t>
+        </is>
+      </c>
+      <c r="D68" s="37" t="inlineStr">
+        <is>
+          <t>चूप</t>
+        </is>
+      </c>
+      <c r="E68" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F68" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G68" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «चुप» -&gt; «चूप»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H68" s="35" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I68" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="B69" s="36" t="inlineStr">
+        <is>
+          <t>tum_x</t>
+        </is>
+      </c>
+      <c r="C69" s="36" t="inlineStr">
+        <is>
+          <t>tum_x.ogg</t>
+        </is>
+      </c>
+      <c r="D69" s="37" t="inlineStr">
+        <is>
+          <t>तूम</t>
+        </is>
+      </c>
+      <c r="E69" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F69" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G69" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «तुम» -&gt; «तूम»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H69" s="35" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I69" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="B70" s="36" t="inlineStr">
+        <is>
+          <t>madhu_x</t>
+        </is>
+      </c>
+      <c r="C70" s="36" t="inlineStr">
+        <is>
+          <t>madhu_x.ogg</t>
+        </is>
+      </c>
+      <c r="D70" s="37" t="inlineStr">
+        <is>
+          <t>मधू</t>
+        </is>
+      </c>
+      <c r="E70" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F70" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G70" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «मधु» -&gt; «मधू»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H70" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I70" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="35" t="n">
+        <v>67</v>
+      </c>
+      <c r="B71" s="36" t="inlineStr">
+        <is>
+          <t>sui_x</t>
+        </is>
+      </c>
+      <c r="C71" s="36" t="inlineStr">
+        <is>
+          <t>sui_x.ogg</t>
+        </is>
+      </c>
+      <c r="D71" s="37" t="inlineStr">
+        <is>
+          <t>सूई</t>
+        </is>
+      </c>
+      <c r="E71" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F71" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G71" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «सुई» -&gt; «सूई»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H71" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I71" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="35" t="n">
+        <v>68</v>
+      </c>
+      <c r="B72" s="36" t="inlineStr">
+        <is>
+          <t>kutta_x</t>
+        </is>
+      </c>
+      <c r="C72" s="36" t="inlineStr">
+        <is>
+          <t>kutta_x.ogg</t>
+        </is>
+      </c>
+      <c r="D72" s="37" t="inlineStr">
+        <is>
+          <t>कूत्ता</t>
+        </is>
+      </c>
+      <c r="E72" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F72" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G72" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «कुत्ता» -&gt; «कूत्ता»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H72" s="35" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I72" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="35" t="n">
+        <v>69</v>
+      </c>
+      <c r="B73" s="36" t="inlineStr">
+        <is>
+          <t>gulab_x</t>
+        </is>
+      </c>
+      <c r="C73" s="36" t="inlineStr">
+        <is>
+          <t>gulab_x.ogg</t>
+        </is>
+      </c>
+      <c r="D73" s="37" t="inlineStr">
+        <is>
+          <t>गूलाब</t>
+        </is>
+      </c>
+      <c r="E73" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F73" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G73" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «गुलाब» -&gt; «गूलाब»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H73" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I73" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="35" t="n">
+        <v>70</v>
+      </c>
+      <c r="B74" s="36" t="inlineStr">
+        <is>
+          <t>subah_x</t>
+        </is>
+      </c>
+      <c r="C74" s="36" t="inlineStr">
+        <is>
+          <t>subah_x.ogg</t>
+        </is>
+      </c>
+      <c r="D74" s="37" t="inlineStr">
+        <is>
+          <t>सूबह</t>
+        </is>
+      </c>
+      <c r="E74" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F74" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G74" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «सुबह» -&gt; «सूबह»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H74" s="35" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I74" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="35" t="n">
+        <v>71</v>
+      </c>
+      <c r="B75" s="36" t="inlineStr">
+        <is>
+          <t>dukan_x</t>
+        </is>
+      </c>
+      <c r="C75" s="36" t="inlineStr">
+        <is>
+          <t>dukan_x.ogg</t>
+        </is>
+      </c>
+      <c r="D75" s="37" t="inlineStr">
+        <is>
+          <t>दूकान</t>
+        </is>
+      </c>
+      <c r="E75" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F75" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G75" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «दुकान» -&gt; «दूकान»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H75" s="35" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I75" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="35" t="n">
+        <v>72</v>
+      </c>
+      <c r="B76" s="36" t="inlineStr">
+        <is>
+          <t>mukut_x</t>
+        </is>
+      </c>
+      <c r="C76" s="36" t="inlineStr">
+        <is>
+          <t>mukut_x.ogg</t>
+        </is>
+      </c>
+      <c r="D76" s="37" t="inlineStr">
+        <is>
+          <t>मूकुट</t>
+        </is>
+      </c>
+      <c r="E76" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F76" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G76" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «मुकुट» -&gt; «मूकुट»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H76" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I76" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="35" t="n">
+        <v>73</v>
+      </c>
+      <c r="B77" s="36" t="inlineStr">
+        <is>
+          <t>gudiya_x</t>
+        </is>
+      </c>
+      <c r="C77" s="36" t="inlineStr">
+        <is>
+          <t>gudiya_x.ogg</t>
+        </is>
+      </c>
+      <c r="D77" s="37" t="inlineStr">
+        <is>
+          <t>गूड़िया</t>
+        </is>
+      </c>
+      <c r="E77" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F77" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G77" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «गुड़िया» -&gt; «गूड़िया»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H77" s="35" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I77" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="35" t="n">
+        <v>74</v>
+      </c>
+      <c r="B78" s="36" t="inlineStr">
+        <is>
+          <t>jamun_x</t>
+        </is>
+      </c>
+      <c r="C78" s="36" t="inlineStr">
+        <is>
+          <t>jamun_x.ogg</t>
+        </is>
+      </c>
+      <c r="D78" s="37" t="inlineStr">
+        <is>
+          <t>जामून</t>
+        </is>
+      </c>
+      <c r="E78" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F78" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G78" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «जामुन» -&gt; «जामून»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H78" s="35" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I78" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="B79" s="36" t="inlineStr">
+        <is>
+          <t>bulbul_x</t>
+        </is>
+      </c>
+      <c r="C79" s="36" t="inlineStr">
+        <is>
+          <t>bulbul_x.ogg</t>
+        </is>
+      </c>
+      <c r="D79" s="37" t="inlineStr">
+        <is>
+          <t>बूलबुल</t>
+        </is>
+      </c>
+      <c r="E79" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F79" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G79" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «बुलबुल» -&gt; «बूलबुल»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H79" s="35" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="I79" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="35" t="n">
+        <v>76</v>
+      </c>
+      <c r="B80" s="36" t="inlineStr">
+        <is>
+          <t>kursi_x</t>
+        </is>
+      </c>
+      <c r="C80" s="36" t="inlineStr">
+        <is>
+          <t>kursi_x.ogg</t>
+        </is>
+      </c>
+      <c r="D80" s="37" t="inlineStr">
+        <is>
+          <t>कूर्सी</t>
+        </is>
+      </c>
+      <c r="E80" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F80" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G80" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «कुर्सी» -&gt; «कूर्सी»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H80" s="35" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="I80" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="35" t="n">
+        <v>77</v>
+      </c>
+      <c r="B81" s="36" t="inlineStr">
+        <is>
+          <t>pustak_x</t>
+        </is>
+      </c>
+      <c r="C81" s="36" t="inlineStr">
+        <is>
+          <t>pustak_x.ogg</t>
+        </is>
+      </c>
+      <c r="D81" s="37" t="inlineStr">
+        <is>
+          <t>पूस्तक</t>
+        </is>
+      </c>
+      <c r="E81" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F81" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G81" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «पुस्तक» -&gt; «पूस्तक»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H81" s="35" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="I81" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="35" t="n">
+        <v>78</v>
+      </c>
+      <c r="B82" s="36" t="inlineStr">
+        <is>
+          <t>chuhiya_x</t>
+        </is>
+      </c>
+      <c r="C82" s="36" t="inlineStr">
+        <is>
+          <t>chuhiya_x.ogg</t>
+        </is>
+      </c>
+      <c r="D82" s="37" t="inlineStr">
+        <is>
+          <t>चूहिया</t>
+        </is>
+      </c>
+      <c r="E82" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F82" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G82" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «चुहिया» -&gt; «चूहिया»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H82" s="35" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="I82" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="35" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="36" t="inlineStr">
+        <is>
+          <t>murli_x</t>
+        </is>
+      </c>
+      <c r="C83" s="36" t="inlineStr">
+        <is>
+          <t>murli_x.ogg</t>
+        </is>
+      </c>
+      <c r="D83" s="37" t="inlineStr">
+        <is>
+          <t>मूरली</t>
+        </is>
+      </c>
+      <c r="E83" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F83" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G83" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «मुरली» -&gt; «मूरली»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H83" s="35" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="I83" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="35" t="n">
+        <v>80</v>
+      </c>
+      <c r="B84" s="36" t="inlineStr">
+        <is>
+          <t>budhiya_x</t>
+        </is>
+      </c>
+      <c r="C84" s="36" t="inlineStr">
+        <is>
+          <t>budhiya_x.ogg</t>
+        </is>
+      </c>
+      <c r="D84" s="37" t="inlineStr">
+        <is>
+          <t>बूढ़िया</t>
+        </is>
+      </c>
+      <c r="E84" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F84" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G84" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «बुढ़िया» -&gt; «बूढ़िया»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H84" s="35" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="I84" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="35" t="n">
+        <v>81</v>
+      </c>
+      <c r="B85" s="36" t="inlineStr">
+        <is>
+          <t>surahi_x</t>
+        </is>
+      </c>
+      <c r="C85" s="36" t="inlineStr">
+        <is>
+          <t>surahi_x.ogg</t>
+        </is>
+      </c>
+      <c r="D85" s="37" t="inlineStr">
+        <is>
+          <t>सूराही</t>
+        </is>
+      </c>
+      <c r="E85" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F85" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G85" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «सुराही» -&gt; «सूराही»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H85" s="35" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="I85" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="35" t="n">
+        <v>82</v>
+      </c>
+      <c r="B86" s="36" t="inlineStr">
+        <is>
+          <t>kulhadi_x</t>
+        </is>
+      </c>
+      <c r="C86" s="36" t="inlineStr">
+        <is>
+          <t>kulhadi_x.ogg</t>
+        </is>
+      </c>
+      <c r="D86" s="37" t="inlineStr">
+        <is>
+          <t>कूल्हाड़ी</t>
+        </is>
+      </c>
+      <c r="E86" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F86" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G86" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «कुल्हाड़ी» -&gt; «कूल्हाड़ी»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H86" s="35" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I86" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="35" t="n">
+        <v>83</v>
+      </c>
+      <c r="B87" s="36" t="inlineStr">
+        <is>
+          <t>phool_x</t>
+        </is>
+      </c>
+      <c r="C87" s="36" t="inlineStr">
+        <is>
+          <t>phool_x.ogg</t>
+        </is>
+      </c>
+      <c r="D87" s="37" t="inlineStr">
+        <is>
+          <t>फुल</t>
+        </is>
+      </c>
+      <c r="E87" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F87" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G87" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «फूल» -&gt; «फुल»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H87" s="35" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I87" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="35" t="n">
+        <v>84</v>
+      </c>
+      <c r="B88" s="36" t="inlineStr">
+        <is>
+          <t>jhoola_x</t>
+        </is>
+      </c>
+      <c r="C88" s="36" t="inlineStr">
+        <is>
+          <t>jhoola_x.ogg</t>
+        </is>
+      </c>
+      <c r="D88" s="37" t="inlineStr">
+        <is>
+          <t>झुला</t>
+        </is>
+      </c>
+      <c r="E88" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F88" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G88" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «झूला» -&gt; «झुला»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H88" s="35" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="I88" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="35" t="n">
+        <v>85</v>
+      </c>
+      <c r="B89" s="36" t="inlineStr">
+        <is>
+          <t>doodh_x</t>
+        </is>
+      </c>
+      <c r="C89" s="36" t="inlineStr">
+        <is>
+          <t>doodh_x.ogg</t>
+        </is>
+      </c>
+      <c r="D89" s="37" t="inlineStr">
+        <is>
+          <t>दुध</t>
+        </is>
+      </c>
+      <c r="E89" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F89" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G89" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «दूध» -&gt; «दुध»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H89" s="35" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="I89" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="35" t="n">
+        <v>86</v>
+      </c>
+      <c r="B90" s="36" t="inlineStr">
+        <is>
+          <t>sooraj_x</t>
+        </is>
+      </c>
+      <c r="C90" s="36" t="inlineStr">
+        <is>
+          <t>sooraj_x.ogg</t>
+        </is>
+      </c>
+      <c r="D90" s="37" t="inlineStr">
+        <is>
+          <t>सुरज</t>
+        </is>
+      </c>
+      <c r="E90" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F90" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G90" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «सूरज» -&gt; «सुरज»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H90" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I90" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="35" t="n">
+        <v>87</v>
+      </c>
+      <c r="B91" s="36" t="inlineStr">
+        <is>
+          <t>mooli_x</t>
+        </is>
+      </c>
+      <c r="C91" s="36" t="inlineStr">
+        <is>
+          <t>mooli_x.ogg</t>
+        </is>
+      </c>
+      <c r="D91" s="37" t="inlineStr">
+        <is>
+          <t>मुली</t>
+        </is>
+      </c>
+      <c r="E91" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F91" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G91" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «मूली» -&gt; «मुली»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H91" s="35" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="I91" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="35" t="n">
+        <v>88</v>
+      </c>
+      <c r="B92" s="36" t="inlineStr">
+        <is>
+          <t>chooha_x</t>
+        </is>
+      </c>
+      <c r="C92" s="36" t="inlineStr">
+        <is>
+          <t>chooha_x.ogg</t>
+        </is>
+      </c>
+      <c r="D92" s="37" t="inlineStr">
+        <is>
+          <t>चुहा</t>
+        </is>
+      </c>
+      <c r="E92" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F92" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G92" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «चूहा» -&gt; «चुहा»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H92" s="35" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I92" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="35" t="n">
+        <v>89</v>
+      </c>
+      <c r="B93" s="36" t="inlineStr">
+        <is>
+          <t>joota_x</t>
+        </is>
+      </c>
+      <c r="C93" s="36" t="inlineStr">
+        <is>
+          <t>joota_x.ogg</t>
+        </is>
+      </c>
+      <c r="D93" s="37" t="inlineStr">
+        <is>
+          <t>जुता</t>
+        </is>
+      </c>
+      <c r="E93" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F93" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G93" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «जूता» -&gt; «जुता»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H93" s="35" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="I93" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="35" t="n">
+        <v>90</v>
+      </c>
+      <c r="B94" s="36" t="inlineStr">
+        <is>
+          <t>bhaloo_x</t>
+        </is>
+      </c>
+      <c r="C94" s="36" t="inlineStr">
+        <is>
+          <t>bhaloo_x.ogg</t>
+        </is>
+      </c>
+      <c r="D94" s="37" t="inlineStr">
+        <is>
+          <t>भालु</t>
+        </is>
+      </c>
+      <c r="E94" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F94" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G94" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «भालू» -&gt; «भालु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H94" s="35" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="I94" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="35" t="n">
+        <v>91</v>
+      </c>
+      <c r="B95" s="36" t="inlineStr">
+        <is>
+          <t>kabootar_x</t>
+        </is>
+      </c>
+      <c r="C95" s="36" t="inlineStr">
+        <is>
+          <t>kabootar_x.ogg</t>
+        </is>
+      </c>
+      <c r="D95" s="37" t="inlineStr">
+        <is>
+          <t>कबुतर</t>
+        </is>
+      </c>
+      <c r="E95" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F95" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G95" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «कबूतर» -&gt; «कबुतर»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H95" s="35" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I95" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="B96" s="36" t="inlineStr">
+        <is>
+          <t>aaloo_x</t>
+        </is>
+      </c>
+      <c r="C96" s="36" t="inlineStr">
+        <is>
+          <t>aaloo_x.ogg</t>
+        </is>
+      </c>
+      <c r="D96" s="37" t="inlineStr">
+        <is>
+          <t>आलु</t>
+        </is>
+      </c>
+      <c r="E96" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F96" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G96" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «आलू» -&gt; «आलु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H96" s="35" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="I96" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="35" t="n">
+        <v>93</v>
+      </c>
+      <c r="B97" s="36" t="inlineStr">
+        <is>
+          <t>chaakoo_x</t>
+        </is>
+      </c>
+      <c r="C97" s="36" t="inlineStr">
+        <is>
+          <t>chaakoo_x.ogg</t>
+        </is>
+      </c>
+      <c r="D97" s="37" t="inlineStr">
+        <is>
+          <t>चाकु</t>
+        </is>
+      </c>
+      <c r="E97" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F97" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G97" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «चाकू» -&gt; «चाकु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H97" s="35" t="n"/>
+      <c r="I97" s="40" t="inlineStr">
+        <is>
+          <t>MISSING - record</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="35" t="n">
+        <v>94</v>
+      </c>
+      <c r="B98" s="36" t="inlineStr">
+        <is>
+          <t>dhoop_x</t>
+        </is>
+      </c>
+      <c r="C98" s="36" t="inlineStr">
+        <is>
+          <t>dhoop_x.ogg</t>
+        </is>
+      </c>
+      <c r="D98" s="37" t="inlineStr">
+        <is>
+          <t>धुप</t>
+        </is>
+      </c>
+      <c r="E98" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F98" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G98" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «धूप» -&gt; «धुप»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H98" s="35" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I98" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="35" t="n">
+        <v>95</v>
+      </c>
+      <c r="B99" s="36" t="inlineStr">
+        <is>
+          <t>choodi_x</t>
+        </is>
+      </c>
+      <c r="C99" s="36" t="inlineStr">
+        <is>
+          <t>choodi_x.ogg</t>
+        </is>
+      </c>
+      <c r="D99" s="37" t="inlineStr">
+        <is>
+          <t>चुड़ी</t>
+        </is>
+      </c>
+      <c r="E99" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F99" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G99" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «चूड़ी» -&gt; «चुड़ी»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H99" s="35" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I99" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="35" t="n">
+        <v>96</v>
+      </c>
+      <c r="B100" s="36" t="inlineStr">
+        <is>
+          <t>jhooth_x</t>
+        </is>
+      </c>
+      <c r="C100" s="36" t="inlineStr">
+        <is>
+          <t>jhooth_x.ogg</t>
+        </is>
+      </c>
+      <c r="D100" s="37" t="inlineStr">
+        <is>
+          <t>झुठ</t>
+        </is>
+      </c>
+      <c r="E100" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F100" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G100" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «झूठ» -&gt; «झुठ»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H100" s="35" t="n"/>
+      <c r="I100" s="40" t="inlineStr">
+        <is>
+          <t>MISSING - record</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="35" t="n">
+        <v>97</v>
+      </c>
+      <c r="B101" s="36" t="inlineStr">
+        <is>
+          <t>pooja_x</t>
+        </is>
+      </c>
+      <c r="C101" s="36" t="inlineStr">
+        <is>
+          <t>pooja_x.ogg</t>
+        </is>
+      </c>
+      <c r="D101" s="37" t="inlineStr">
+        <is>
+          <t>पुजा</t>
+        </is>
+      </c>
+      <c r="E101" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F101" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G101" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «पूजा» -&gt; «पुजा»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H101" s="35" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="I101" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="35" t="n">
+        <v>98</v>
+      </c>
+      <c r="B102" s="36" t="inlineStr">
+        <is>
+          <t>kooda_x</t>
+        </is>
+      </c>
+      <c r="C102" s="36" t="inlineStr">
+        <is>
+          <t>kooda_x.ogg</t>
+        </is>
+      </c>
+      <c r="D102" s="37" t="inlineStr">
+        <is>
+          <t>कुड़ा</t>
+        </is>
+      </c>
+      <c r="E102" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F102" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G102" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «कूड़ा» -&gt; «कुड़ा»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H102" s="35" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I102" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="35" t="n">
+        <v>99</v>
+      </c>
+      <c r="B103" s="36" t="inlineStr">
+        <is>
+          <t>bhookh_x</t>
+        </is>
+      </c>
+      <c r="C103" s="36" t="inlineStr">
+        <is>
+          <t>bhookh_x.ogg</t>
+        </is>
+      </c>
+      <c r="D103" s="37" t="inlineStr">
+        <is>
+          <t>भुख</t>
+        </is>
+      </c>
+      <c r="E103" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F103" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G103" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «भूख» -&gt; «भुख»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H103" s="35" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="I103" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" s="36" t="inlineStr">
+        <is>
+          <t>angoor_x</t>
+        </is>
+      </c>
+      <c r="C104" s="36" t="inlineStr">
+        <is>
+          <t>angoor_x.ogg</t>
+        </is>
+      </c>
+      <c r="D104" s="37" t="inlineStr">
+        <is>
+          <t>अंगुर</t>
+        </is>
+      </c>
+      <c r="E104" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F104" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G104" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «अंगूर» -&gt; «अंगुर»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H104" s="35" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I104" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="35" t="n">
+        <v>101</v>
+      </c>
+      <c r="B105" s="36" t="inlineStr">
+        <is>
+          <t>tarbooj_x</t>
+        </is>
+      </c>
+      <c r="C105" s="36" t="inlineStr">
+        <is>
+          <t>tarbooj_x.ogg</t>
+        </is>
+      </c>
+      <c r="D105" s="37" t="inlineStr">
+        <is>
+          <t>तरबुज</t>
+        </is>
+      </c>
+      <c r="E105" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F105" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G105" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «तरबूज» -&gt; «तरबुज»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H105" s="35" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="I105" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="35" t="n">
+        <v>102</v>
+      </c>
+      <c r="B106" s="36" t="inlineStr">
+        <is>
+          <t>neemboo_x</t>
+        </is>
+      </c>
+      <c r="C106" s="36" t="inlineStr">
+        <is>
+          <t>neemboo_x.ogg</t>
+        </is>
+      </c>
+      <c r="D106" s="37" t="inlineStr">
+        <is>
+          <t>नींबु</t>
+        </is>
+      </c>
+      <c r="E106" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F106" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G106" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «नींबू» -&gt; «नींबु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H106" s="35" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="I106" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="35" t="n">
+        <v>103</v>
+      </c>
+      <c r="B107" s="36" t="inlineStr">
+        <is>
+          <t>kaaju_x</t>
+        </is>
+      </c>
+      <c r="C107" s="36" t="inlineStr">
+        <is>
+          <t>kaaju_x.ogg</t>
+        </is>
+      </c>
+      <c r="D107" s="37" t="inlineStr">
+        <is>
+          <t>काजु</t>
+        </is>
+      </c>
+      <c r="E107" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F107" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G107" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «काजू» -&gt; «काजु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H107" s="35" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I107" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="35" t="n">
+        <v>104</v>
+      </c>
+      <c r="B108" s="36" t="inlineStr">
+        <is>
+          <t>taraaju_x</t>
+        </is>
+      </c>
+      <c r="C108" s="36" t="inlineStr">
+        <is>
+          <t>taraaju_x.ogg</t>
+        </is>
+      </c>
+      <c r="D108" s="37" t="inlineStr">
+        <is>
+          <t>तराजु</t>
+        </is>
+      </c>
+      <c r="E108" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F108" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G108" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «तराजू» -&gt; «तराजु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H108" s="35" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="I108" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="35" t="n">
+        <v>105</v>
+      </c>
+      <c r="B109" s="36" t="inlineStr">
+        <is>
+          <t>lattoo_x</t>
+        </is>
+      </c>
+      <c r="C109" s="36" t="inlineStr">
+        <is>
+          <t>lattoo_x.ogg</t>
+        </is>
+      </c>
+      <c r="D109" s="37" t="inlineStr">
+        <is>
+          <t>लट्टु</t>
+        </is>
+      </c>
+      <c r="E109" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F109" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G109" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «लट्टू» -&gt; «लट्टु»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H109" s="35" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I109" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="35" t="n">
+        <v>106</v>
+      </c>
+      <c r="B110" s="36" t="inlineStr">
+        <is>
+          <t>bandook_x</t>
+        </is>
+      </c>
+      <c r="C110" s="36" t="inlineStr">
+        <is>
+          <t>bandook_x.ogg</t>
+        </is>
+      </c>
+      <c r="D110" s="37" t="inlineStr">
+        <is>
+          <t>बंदुक</t>
+        </is>
+      </c>
+      <c r="E110" s="36" t="inlineStr">
+        <is>
+          <t>Twin (wrong option)</t>
+        </is>
+      </c>
+      <c r="F110" s="38" t="inlineStr">
+        <is>
+          <t>the other matra</t>
+        </is>
+      </c>
+      <c r="G110" s="39" t="inlineStr">
+        <is>
+          <t>The WRONG option of a minimal pair (one matra swapped, «बंदूक» -&gt; «बंदुक»). Read only when that pair comes back after a first mistake. TTS PLACEHOLDER - record.</t>
+        </is>
+      </c>
+      <c r="H110" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I110" s="36" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:I64"/>
+  <autoFilter ref="A4:I110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3237,229 +5234,229 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="35" t="inlineStr"/>
+      <c r="A2" s="41" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="inlineStr">
+      <c r="A3" s="42" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B3" s="37" t="inlineStr">
+      <c r="B3" s="43" t="inlineStr">
         <is>
           <t>The runner game on page 17 only. The rest of the lesson has its own VO in assets/Audio/.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Clips</t>
         </is>
       </c>
-      <c r="B4" s="37" t="inlineStr">
+      <c r="B4" s="43" t="inlineStr">
         <is>
           <t>60 in total: 14 lines (13 used, 1 unused) + 22 words with छोटी उ + 24 words with बड़ी ऊ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="42" t="inlineStr">
         <is>
           <t>Folder</t>
         </is>
       </c>
-      <c r="B5" s="37" t="inlineStr">
+      <c r="B5" s="43" t="inlineStr">
         <is>
           <t>3_CURRENT_BUILD/assets/MatraRunner/voice/&lt;Audio ID&gt;.ogg  - the file name is the Audio ID; the game finds clips by it</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>Voice</t>
         </is>
       </c>
-      <c r="B6" s="37" t="inlineStr">
+      <c r="B6" s="43" t="inlineStr">
         <is>
           <t>Recorded VO supplied 2026-09-29 (sources: 1_SPEC/game_art_src/runner_voice/source_wav/). Keep ONE narrator for every clip. Previous Gemini TTS (Leda) takes are kept in runner_voice/takes_gemini_leda_r79/.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="inlineStr">
+      <c r="A7" s="42" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="B7" s="37" t="inlineStr">
+      <c r="B7" s="43" t="inlineStr">
         <is>
           <t>Deliver WAV (mono, 24 kHz or higher), named &lt;Audio ID&gt;.wav. 1_SPEC/prepare_runner_voice.py then trims the silence, levels to -16 LUFS (the lesson's VO level, peaks limited at -3 dBFS) and encodes Ogg Vorbis mono 24 kHz for the game.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>Register</t>
         </is>
       </c>
-      <c r="B8" s="37" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>आप form throughout (पकड़िए / देखिए / कीजिए) - never तुम.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="42" t="inlineStr">
         <is>
           <t>Words</t>
         </is>
       </c>
-      <c r="B9" s="37" t="inlineStr">
+      <c r="B9" s="43" t="inlineStr">
         <is>
           <t>Say each word on its own, plainly, as a word - no carrier sentence, no question tone. Keep the matra's length true: छोटी उ short (पुल, गुड़), बड़ी ऊ long (फूल, दूध) - but do not stretch it for effect.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
         <is>
           <t>Re-recording</t>
         </is>
       </c>
-      <c r="B10" s="37" t="inlineStr">
+      <c r="B10" s="43" t="inlineStr">
         <is>
           <t>Keep the same file name. The build stamps the game's audio with a content hash (?v=...), so a new take reaches browsers after the next deploy.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="35" t="inlineStr"/>
+      <c r="A11" s="41" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="35" t="inlineStr">
+      <c r="A12" s="41" t="inlineStr">
         <is>
           <t>What plays when</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="inlineStr">
+      <c r="A13" s="42" t="inlineStr">
         <is>
           <t>1. Game page opens</t>
         </is>
       </c>
-      <c r="B13" s="37" t="inlineStr">
+      <c r="B13" s="43" t="inlineStr">
         <is>
           <t>The lesson says its own instruction (NOT in this manifest - lesson clip assets/Audio/vo_mg_prompt.ogg): «अब एक खेल! ऊपर दी गई मात्रा वाले शब्द के द्वार से निकलिए।»</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="A14" s="42" t="inlineStr">
         <is>
           <t>2. Tutorial (first time)</t>
         </is>
       </c>
-      <c r="B14" s="37" t="inlineStr">
+      <c r="B14" s="43" t="inlineStr">
         <is>
           <t>tut_lane, tut_jump, tut_slide - each as the run stops in front of its obstacle - then tut_go</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="36" t="inlineStr">
+      <c r="A15" s="42" t="inlineStr">
         <is>
           <t>3. Level 1 goal</t>
         </is>
       </c>
-      <c r="B15" s="37" t="inlineStr">
+      <c r="B15" s="43" t="inlineStr">
         <is>
           <t>goal_uu - «बड़ी ऊ की मात्रा वाले शब्द पकड़िए।»</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="36" t="inlineStr">
+      <c r="A16" s="42" t="inlineStr">
         <is>
           <t>4. Each pair of word orbs</t>
         </is>
       </c>
-      <c r="B16" s="37" t="inlineStr">
-        <is>
-          <t>Only the target word, as the pair comes near (after a clear pause).</t>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Nothing - the child reads the words (r115).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="36" t="inlineStr">
+      <c r="A17" s="42" t="inlineStr">
         <is>
           <t>5. Correct orb</t>
         </is>
       </c>
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B17" s="43" t="inlineStr">
         <is>
           <t>right - «शाबाश!»</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="36" t="inlineStr">
+      <c r="A18" s="42" t="inlineStr">
         <is>
           <t>6. Wrong orb</t>
         </is>
       </c>
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>wrong + correct_is + the correct word - «फिर से देखिए। सही शब्द है &lt;शब्द&gt;»</t>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>wrong - «फिर से देखिए।»; the pair comes back: after 1 mistake both words are read, after 2 the right word</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="36" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>7. Obstacle hit</t>
         </is>
       </c>
-      <c r="B19" s="37" t="inlineStr">
+      <c r="B19" s="43" t="inlineStr">
         <is>
           <t>hit - «अरे! ध्यान से।»</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="36" t="inlineStr">
+      <c r="A20" s="42" t="inlineStr">
         <is>
           <t>8. Level ends</t>
         </is>
       </c>
-      <c r="B20" s="37" t="inlineStr">
+      <c r="B20" s="43" t="inlineStr">
         <is>
           <t>Screen blurs, chime, then level_next + next goal - «वाह! अब इस लेवल को पार कीजिए।» «छोटी उ की मात्रा वाले शब्द पकड़िए।»</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="36" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>9. All hearts lost</t>
         </is>
       </c>
-      <c r="B21" s="37" t="inlineStr">
+      <c r="B21" s="43" t="inlineStr">
         <is>
           <t>retry - «कोई बात नहीं, फिर से कोशिश कीजिए।», then the level restarts</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="36" t="inlineStr">
+      <c r="A22" s="42" t="inlineStr">
         <is>
           <t>10. Game finished</t>
         </is>
       </c>
-      <c r="B22" s="37" t="inlineStr">
+      <c r="B22" s="43" t="inlineStr">
         <is>
           <t>win - «शाबाश! आपने सारे शब्द पकड़ लिए!»</t>
         </is>

</xml_diff>